<commit_message>
Minor changes based on feedback from Peter G.
</commit_message>
<xml_diff>
--- a/data/phi_data_combined.xlsx
+++ b/data/phi_data_combined.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carolinkilian/Desktop/Research projects/Public Health Index/Github/Public-Health-Index/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B811D35-B7F3-374E-858E-2B0091F3559D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E3CA47-6DBE-7C40-BC12-766826A8D584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{07406E1C-1769-574D-9B9C-B78BFD08E78B}"/>
   </bookViews>
@@ -3991,7 +3991,7 @@
         <v>72</v>
       </c>
       <c r="C146" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D146" t="s">
         <v>31</v>
@@ -4014,7 +4014,7 @@
         <v>72</v>
       </c>
       <c r="C147" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D147" t="s">
         <v>31</v>
@@ -4037,7 +4037,7 @@
         <v>72</v>
       </c>
       <c r="C148" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D148" t="s">
         <v>31</v>
@@ -4060,7 +4060,7 @@
         <v>72</v>
       </c>
       <c r="C149" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D149" t="s">
         <v>31</v>
@@ -4083,7 +4083,7 @@
         <v>72</v>
       </c>
       <c r="C150" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D150" t="s">
         <v>31</v>
@@ -4106,7 +4106,7 @@
         <v>72</v>
       </c>
       <c r="C151" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D151" t="s">
         <v>31</v>
@@ -4129,7 +4129,7 @@
         <v>72</v>
       </c>
       <c r="C152" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D152" t="s">
         <v>31</v>
@@ -4152,7 +4152,7 @@
         <v>72</v>
       </c>
       <c r="C153" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D153" t="s">
         <v>31</v>
@@ -4175,7 +4175,7 @@
         <v>72</v>
       </c>
       <c r="C154" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D154" t="s">
         <v>31</v>
@@ -4198,7 +4198,7 @@
         <v>72</v>
       </c>
       <c r="C155" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D155" t="s">
         <v>31</v>
@@ -4221,7 +4221,7 @@
         <v>72</v>
       </c>
       <c r="C156" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D156" t="s">
         <v>31</v>
@@ -4244,7 +4244,7 @@
         <v>72</v>
       </c>
       <c r="C157" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D157" t="s">
         <v>31</v>
@@ -4267,7 +4267,7 @@
         <v>72</v>
       </c>
       <c r="C158" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D158" t="s">
         <v>31</v>
@@ -4290,7 +4290,7 @@
         <v>72</v>
       </c>
       <c r="C159" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D159" t="s">
         <v>31</v>
@@ -4313,7 +4313,7 @@
         <v>72</v>
       </c>
       <c r="C160" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D160" t="s">
         <v>31</v>
@@ -4336,7 +4336,7 @@
         <v>72</v>
       </c>
       <c r="C161" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D161" t="s">
         <v>31</v>
@@ -4359,7 +4359,7 @@
         <v>72</v>
       </c>
       <c r="C162" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D162" t="s">
         <v>31</v>
@@ -4382,7 +4382,7 @@
         <v>72</v>
       </c>
       <c r="C163" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="D163" t="s">
         <v>31</v>

</xml_diff>